<commit_message>
Update: Added 4 new charts (total 10) and updated dashboard, reports
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -16,9 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0&quot; Days&quot;"/>
+    <numFmt numFmtId="167" formatCode="0&quot; Days&quot;"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -176,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -242,6 +244,21 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -326,7 +343,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>35</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5715000" cy="3429000"/>
@@ -351,7 +368,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>35</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5715000" cy="3429000"/>
@@ -376,7 +393,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>47</row>
+      <row>55</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5715000" cy="3429000"/>
@@ -401,7 +418,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>47</row>
+      <row>55</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5715000" cy="3429000"/>
@@ -412,6 +429,156 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>75</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5715000" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>75</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5715000" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>95</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5715000" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>95</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5715000" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>115</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5715000" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>115</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5715000" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -714,7 +881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -726,9 +893,9 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="4" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
     <col width="4" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
@@ -900,7 +1067,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
+    <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Month</t>
@@ -967,7 +1134,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
+    <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
           <t>2017-09</t>
@@ -1019,7 +1186,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
+    <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>2017-10</t>
@@ -1071,7 +1238,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
+    <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
           <t>2017-11</t>
@@ -1123,7 +1290,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
+    <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>2017-12</t>
@@ -1175,7 +1342,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1">
+    <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
           <t>2018-01</t>
@@ -1227,7 +1394,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
+    <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
           <t>2018-02</t>
@@ -1280,7 +1447,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1">
+    <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
           <t>2018-03</t>
@@ -1320,7 +1487,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
+    <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
           <t>2018-04</t>
@@ -1360,7 +1527,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1">
+    <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
           <t>2018-05</t>
@@ -1400,7 +1567,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1">
+    <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
           <t>2018-06</t>
@@ -1440,7 +1607,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1">
+    <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
           <t>2018-07</t>
@@ -1482,7 +1649,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1">
+    <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
           <t>2018-08</t>
@@ -1498,7 +1665,7 @@
         <v>132.2006073820277</v>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
+    <row r="24">
       <c r="A24" s="22" t="inlineStr">
         <is>
           <t>Total/Average</t>
@@ -1517,14 +1684,251 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1"/>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>PERFORMANCE VISUALISATIONS &amp; CHARTS</t>
-        </is>
-      </c>
-    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>Payment Type</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>Payment Value</t>
+        </is>
+      </c>
+      <c r="H25" s="11" t="inlineStr">
+        <is>
+          <t>% Share</t>
+        </is>
+      </c>
+      <c r="J25" s="11" t="inlineStr">
+        <is>
+          <t>Review Rating</t>
+        </is>
+      </c>
+      <c r="K25" s="11" t="inlineStr">
+        <is>
+          <t>Avg Delivery Time</t>
+        </is>
+      </c>
+      <c r="L25" s="11" t="inlineStr">
+        <is>
+          <t>Target (Days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G26" s="13" t="n">
+        <v>9558581.23</v>
+      </c>
+      <c r="H26" s="16">
+        <f>G26/12111199.71</f>
+        <v/>
+      </c>
+      <c r="J26" s="12" t="inlineStr">
+        <is>
+          <t>1 Stars</t>
+        </is>
+      </c>
+      <c r="K26" s="27" t="n">
+        <v>21.45485564304462</v>
+      </c>
+      <c r="L26" s="28" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="F27" s="20" t="inlineStr">
+        <is>
+          <t>Boleto</t>
+        </is>
+      </c>
+      <c r="G27" s="18" t="n">
+        <v>2102613.81</v>
+      </c>
+      <c r="H27" s="21">
+        <f>G27/12111199.71</f>
+        <v/>
+      </c>
+      <c r="J27" s="17" t="inlineStr">
+        <is>
+          <t>1 Stars</t>
+        </is>
+      </c>
+      <c r="K27" s="29" t="n">
+        <v>18.33333333333333</v>
+      </c>
+      <c r="L27" s="30" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>Voucher</t>
+        </is>
+      </c>
+      <c r="G28" s="13" t="n">
+        <v>257267.8</v>
+      </c>
+      <c r="H28" s="16">
+        <f>G28/12111199.71</f>
+        <v/>
+      </c>
+      <c r="J28" s="12" t="inlineStr">
+        <is>
+          <t>2 Stars</t>
+        </is>
+      </c>
+      <c r="K28" s="27" t="n">
+        <v>16.68374558303887</v>
+      </c>
+      <c r="L28" s="28" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="F29" s="20" t="inlineStr">
+        <is>
+          <t>Debit Card</t>
+        </is>
+      </c>
+      <c r="G29" s="18" t="n">
+        <v>192736.87</v>
+      </c>
+      <c r="H29" s="21">
+        <f>G29/12111199.71</f>
+        <v/>
+      </c>
+      <c r="J29" s="17" t="inlineStr">
+        <is>
+          <t>2 Stars</t>
+        </is>
+      </c>
+      <c r="K29" s="29" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="L29" s="30" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="F30" s="25" t="inlineStr">
+        <is>
+          <t>Total Payments</t>
+        </is>
+      </c>
+      <c r="G30" s="26">
+        <f>SUM(G26:G29)</f>
+        <v/>
+      </c>
+      <c r="H30" s="24">
+        <f>SUM(H26:H29)</f>
+        <v/>
+      </c>
+      <c r="J30" s="12" t="inlineStr">
+        <is>
+          <t>3 Stars</t>
+        </is>
+      </c>
+      <c r="K30" s="27" t="n">
+        <v>14.03958919993374</v>
+      </c>
+      <c r="L30" s="28" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="J31" s="17" t="inlineStr">
+        <is>
+          <t>3 Stars</t>
+        </is>
+      </c>
+      <c r="K31" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="L31" s="30" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="J32" s="12" t="inlineStr">
+        <is>
+          <t>3 Stars</t>
+        </is>
+      </c>
+      <c r="K32" s="27" t="n">
+        <v>12.46666666666667</v>
+      </c>
+      <c r="L32" s="28" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="J33" s="17" t="inlineStr">
+        <is>
+          <t>4 Stars</t>
+        </is>
+      </c>
+      <c r="K33" s="29" t="n">
+        <v>11.80522367324257</v>
+      </c>
+      <c r="L33" s="30" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>PERFORMANCE VISUALISATIONS &amp; CHARTS (10 CHARTS REPORT)</t>
+        </is>
+      </c>
+      <c r="J34" s="12" t="inlineStr">
+        <is>
+          <t>4 Stars</t>
+        </is>
+      </c>
+      <c r="K34" s="27" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="L34" s="28" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="J35" s="17" t="inlineStr">
+        <is>
+          <t>5 Stars</t>
+        </is>
+      </c>
+      <c r="K35" s="29" t="n">
+        <v>10.1331256490135</v>
+      </c>
+      <c r="L35" s="30" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="J36" s="22" t="inlineStr">
+        <is>
+          <t>Overall Average</t>
+        </is>
+      </c>
+      <c r="K36" s="31">
+        <f>AVERAGE(K26:K35)</f>
+        <v/>
+      </c>
+      <c r="L36" s="25" t="inlineStr"/>
+    </row>
+    <row r="56" ht="20" customHeight="1"/>
+    <row r="76" ht="20" customHeight="1"/>
+    <row r="96" ht="20" customHeight="1"/>
+    <row r="116" ht="20" customHeight="1"/>
+    <row r="136" ht="20" customHeight="1"/>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="D6:E6"/>

</xml_diff>